<commit_message>
Actualizar Excel al 18/05/2026 y mover boton recargar al cuerpo principal
</commit_message>
<xml_diff>
--- a/stock doina.xlsx
+++ b/stock doina.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Operador\Desktop\claude\proyectos claude\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCDCD45F-8813-466D-B56D-F63DFE36ADEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF962744-AFB6-461B-A3AA-302498899636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="jamon parma" sheetId="6" r:id="rId1"/>
@@ -2187,16 +2187,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2204,6 +2204,55 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="73">
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB8B8B8"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
       <fill>
@@ -4111,55 +4160,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB8B8B8"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4174,48 +4174,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{997CEB9B-2923-4A4C-AA11-BC81F05106FA}" name="Tabla4" displayName="Tabla4" ref="A4:F9" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{997CEB9B-2923-4A4C-AA11-BC81F05106FA}" name="Tabla4" displayName="Tabla4" ref="A4:F9" totalsRowShown="0" headerRowDxfId="72" dataDxfId="70" headerRowBorderDxfId="71">
   <autoFilter ref="A4:F9" xr:uid="{997CEB9B-2923-4A4C-AA11-BC81F05106FA}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{D58044D5-F1AF-4DB2-8E35-D03F06ED2F30}" name="FECHA SALAZON" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{7BA6A8B1-DA5D-4B45-8C2B-5CFC6A42635A}" name="N° LOTE" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{A65DC631-4356-42FE-BD04-2628699A424B}" name="UNIDADES" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{87B1504B-F47D-49DC-9377-CEBE16CAB12E}" name="KILOS" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{9E1C1A0F-CB21-45E7-BD09-CAB2E3270DB5}" name="FECHA TERMINACION" dataDxfId="62">
+    <tableColumn id="1" xr3:uid="{D58044D5-F1AF-4DB2-8E35-D03F06ED2F30}" name="FECHA SALAZON" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{7BA6A8B1-DA5D-4B45-8C2B-5CFC6A42635A}" name="N° LOTE" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{A65DC631-4356-42FE-BD04-2628699A424B}" name="UNIDADES" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{87B1504B-F47D-49DC-9377-CEBE16CAB12E}" name="KILOS" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{9E1C1A0F-CB21-45E7-BD09-CAB2E3270DB5}" name="FECHA TERMINACION" dataDxfId="65">
       <calculatedColumnFormula>+A5+$E$3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EF41C38A-EFC0-47BA-BE9A-B85102F26F51}" name="TAMAÑO" dataDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{EF41C38A-EFC0-47BA-BE9A-B85102F26F51}" name="TAMAÑO" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96560466-FF3B-45A2-8068-CE79B791A8ED}" name="Tabla1" displayName="Tabla1" ref="A4:F106" totalsRowShown="0" headerRowDxfId="60" dataDxfId="58" headerRowBorderDxfId="59" tableBorderDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96560466-FF3B-45A2-8068-CE79B791A8ED}" name="Tabla1" displayName="Tabla1" ref="A4:F106" totalsRowShown="0" headerRowDxfId="63" dataDxfId="61" headerRowBorderDxfId="62" tableBorderDxfId="60">
   <autoFilter ref="A4:F106" xr:uid="{96560466-FF3B-45A2-8068-CE79B791A8ED}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6511CF9D-2ADF-4988-8EC0-2ECED776F414}" name="FECHA SALAZON" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{867E7867-BC82-4A47-8AEB-A01A0AE8E08B}" name="N° LOTE" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{15EEC0A0-3708-46F0-A02A-2CF49ABFDBA5}" name="UNIDADES" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{9C28F57B-D2AC-4B6F-816C-47DFC4579365}" name="KILOS" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{2E00FF43-7F3A-4B3F-BF8A-18C51216D6F9}" name="FECHA TERMINACION" dataDxfId="52">
+    <tableColumn id="1" xr3:uid="{6511CF9D-2ADF-4988-8EC0-2ECED776F414}" name="FECHA SALAZON" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{867E7867-BC82-4A47-8AEB-A01A0AE8E08B}" name="N° LOTE" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{15EEC0A0-3708-46F0-A02A-2CF49ABFDBA5}" name="UNIDADES" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{9C28F57B-D2AC-4B6F-816C-47DFC4579365}" name="KILOS" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{2E00FF43-7F3A-4B3F-BF8A-18C51216D6F9}" name="FECHA TERMINACION" dataDxfId="55">
       <calculatedColumnFormula>IF(F5="CHICO",A5+365,IF(F5="GRANDE",A5+395,IF(F5="EXTRAGRANDE",A5+425,"")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{B5BDD0B9-FAAF-4C0C-97F6-37E3C56DD928}" name="TAMAÑO" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{B5BDD0B9-FAAF-4C0C-97F6-37E3C56DD928}" name="TAMAÑO" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D89E842E-78D6-4D45-A634-F585E354D7F2}" name="Tabla5" displayName="Tabla5" ref="A3:E9" totalsRowShown="0" headerRowDxfId="50" dataDxfId="48" headerRowBorderDxfId="49" tableBorderDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D89E842E-78D6-4D45-A634-F585E354D7F2}" name="Tabla5" displayName="Tabla5" ref="A3:E9" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50">
   <autoFilter ref="A3:E9" xr:uid="{D89E842E-78D6-4D45-A634-F585E354D7F2}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9DB3551A-870D-4AA3-A059-127880751B52}" name="FECHA SALAZON" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{36E854DA-A107-49DF-B87C-CDABC1B2F167}" name="N° LOTE" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{35FA5642-14F6-41B8-B848-2C1A4EE12112}" name="UNIDADES" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{FD4A329C-C457-4315-BFD8-434719CF0367}" name="KILOS" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{6A658D4D-67A5-4565-BEDB-40551CF0CFFA}" name="FECHA TERMINACION" dataDxfId="42">
+    <tableColumn id="1" xr3:uid="{9DB3551A-870D-4AA3-A059-127880751B52}" name="FECHA SALAZON" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{36E854DA-A107-49DF-B87C-CDABC1B2F167}" name="N° LOTE" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{35FA5642-14F6-41B8-B848-2C1A4EE12112}" name="UNIDADES" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{FD4A329C-C457-4315-BFD8-434719CF0367}" name="KILOS" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{6A658D4D-67A5-4565-BEDB-40551CF0CFFA}" name="FECHA TERMINACION" dataDxfId="45">
       <calculatedColumnFormula>+A4+$E$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4224,14 +4224,14 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A4E6FF9D-8420-4520-AAEF-BE0A3744D13A}" name="Tabla6" displayName="Tabla6" ref="A3:E4" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40" tableBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A4E6FF9D-8420-4520-AAEF-BE0A3744D13A}" name="Tabla6" displayName="Tabla6" ref="A3:E4" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43" tableBorderDxfId="42">
   <autoFilter ref="A3:E4" xr:uid="{A4E6FF9D-8420-4520-AAEF-BE0A3744D13A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8095F967-1CCC-455D-9A7A-2669B04AF12E}" name="FECHA SALAZON" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{9E1C92DF-8B52-4616-82A7-B24DD2795650}" name="N° LOTE" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{94498F67-4D78-43F6-86C0-2967C1482004}" name="UNIDADES" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{FCC3F240-403E-44D0-BEA7-F5FB2948CC34}" name="KILOS" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{3CB2134E-2828-40EB-9A0E-BAAA53EE19EB}" name="FECHA TERMINACION" dataDxfId="34">
+    <tableColumn id="1" xr3:uid="{8095F967-1CCC-455D-9A7A-2669B04AF12E}" name="FECHA SALAZON" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{9E1C92DF-8B52-4616-82A7-B24DD2795650}" name="N° LOTE" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{94498F67-4D78-43F6-86C0-2967C1482004}" name="UNIDADES" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{FCC3F240-403E-44D0-BEA7-F5FB2948CC34}" name="KILOS" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{3CB2134E-2828-40EB-9A0E-BAAA53EE19EB}" name="FECHA TERMINACION" dataDxfId="37">
       <calculatedColumnFormula>+A4+$E$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4240,14 +4240,14 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E70BF8AE-2DA7-4419-968E-FCD2889D0CE8}" name="Tabla7" displayName="Tabla7" ref="A3:E7" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E70BF8AE-2DA7-4419-968E-FCD2889D0CE8}" name="Tabla7" displayName="Tabla7" ref="A3:E7" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35" tableBorderDxfId="34">
   <autoFilter ref="A3:E7" xr:uid="{E70BF8AE-2DA7-4419-968E-FCD2889D0CE8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5E72FB8D-1254-4E8D-9446-00C71A68F3B6}" name="FECHA SALAZON" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{5EA7F545-78C8-40AA-ACF6-E7E26E7E00B3}" name="N° LOTE" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{1B33CF51-429F-4B85-8609-965D98BF9B6A}" name="UNIDADES" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{A96D48AC-C488-4426-98D8-239C83A6B753}" name="KILOS" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{7EDC9A92-C330-4FEF-B9BC-9CBF6660DFEF}" name="FECHA TERMINACION" dataDxfId="26">
+    <tableColumn id="1" xr3:uid="{5E72FB8D-1254-4E8D-9446-00C71A68F3B6}" name="FECHA SALAZON" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{5EA7F545-78C8-40AA-ACF6-E7E26E7E00B3}" name="N° LOTE" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{1B33CF51-429F-4B85-8609-965D98BF9B6A}" name="UNIDADES" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{A96D48AC-C488-4426-98D8-239C83A6B753}" name="KILOS" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{7EDC9A92-C330-4FEF-B9BC-9CBF6660DFEF}" name="FECHA TERMINACION" dataDxfId="29">
       <calculatedColumnFormula>+A4+$E$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4256,14 +4256,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{11E65F59-2C08-4860-AE7F-6EBB4BE7AD15}" name="Tabla8" displayName="Tabla8" ref="A3:E5" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" tableBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{11E65F59-2C08-4860-AE7F-6EBB4BE7AD15}" name="Tabla8" displayName="Tabla8" ref="A3:E5" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" tableBorderDxfId="26">
   <autoFilter ref="A3:E5" xr:uid="{11E65F59-2C08-4860-AE7F-6EBB4BE7AD15}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E49E6393-EB0D-4EBB-BE41-9259FBBDBF8E}" name="FECHA SALAZON" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{74526E38-F7AE-4812-85BF-C48944F3BC35}" name="N° LOTE" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{608246E2-511D-44B7-BCD0-18E974B17C49}" name="UNIDADES" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{BA9716F9-56C4-43D7-8635-E3659426BBB2}" name="KILOS" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{D392F03C-5B4C-427D-A148-A053A4B30871}" name="FECHA TERMINACION" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{E49E6393-EB0D-4EBB-BE41-9259FBBDBF8E}" name="FECHA SALAZON" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{74526E38-F7AE-4812-85BF-C48944F3BC35}" name="N° LOTE" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{608246E2-511D-44B7-BCD0-18E974B17C49}" name="UNIDADES" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{BA9716F9-56C4-43D7-8635-E3659426BBB2}" name="KILOS" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{D392F03C-5B4C-427D-A148-A053A4B30871}" name="FECHA TERMINACION" dataDxfId="21">
       <calculatedColumnFormula>+A4+$E$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4272,14 +4272,14 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3C40D0A9-3E05-42AA-BC35-0957ED493BBB}" name="Tabla9" displayName="Tabla9" ref="A3:E27" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3C40D0A9-3E05-42AA-BC35-0957ED493BBB}" name="Tabla9" displayName="Tabla9" ref="A3:E27" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A3:E27" xr:uid="{3C40D0A9-3E05-42AA-BC35-0957ED493BBB}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5E9BE612-58C6-4DC0-B1EE-69AA05A0B4AD}" name="FECHA SALAZON" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{65AFB3AE-A20B-4ADA-BA53-0778B7920450}" name="N° LOTE" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B1ED6BC0-89AE-4280-B231-3B889D85E039}" name="UNIDADES" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{E89CDCA3-58F8-4F3C-A6E8-AD74C095BDF3}" name="KILOS" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{FE11545C-5892-4FF5-9F69-CD83EE14E9C7}" name="FECHA TERMINACION" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{5E9BE612-58C6-4DC0-B1EE-69AA05A0B4AD}" name="FECHA SALAZON" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{65AFB3AE-A20B-4ADA-BA53-0778B7920450}" name="N° LOTE" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{B1ED6BC0-89AE-4280-B231-3B889D85E039}" name="UNIDADES" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{E89CDCA3-58F8-4F3C-A6E8-AD74C095BDF3}" name="KILOS" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{FE11545C-5892-4FF5-9F69-CD83EE14E9C7}" name="FECHA TERMINACION" dataDxfId="13">
       <calculatedColumnFormula>+A4+$E$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4288,23 +4288,23 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{287B2A14-7FAB-4F9D-B0EB-BEBD76034667}" name="Tabla2" displayName="Tabla2" ref="A23:G249" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{287B2A14-7FAB-4F9D-B0EB-BEBD76034667}" name="Tabla2" displayName="Tabla2" ref="A23:G249" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A23:G249" xr:uid="{287B2A14-7FAB-4F9D-B0EB-BEBD76034667}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{208BB7C0-575D-4B00-8DBE-006D1DDA2DC2}" name="Producto" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{DFC7EC60-A2E1-4C2B-9F5F-049C8E21245E}" name="Lote" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{683E82B8-B50D-4767-AA2F-7327EC16B03C}" name="Unidades" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{103F51FD-4980-4385-8737-6C121234FAAE}" name="Kg Bruto" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{1D36A2BF-02B3-4785-8579-39342D79E068}" name="Tara" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{90ECC13E-B58B-4180-8A1A-8808CCF6A5BD}" name="Kg Neto" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{64D76550-4432-4FE0-BDF8-015B9BCBB585}" name="Envasado" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{208BB7C0-575D-4B00-8DBE-006D1DDA2DC2}" name="Producto" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{DFC7EC60-A2E1-4C2B-9F5F-049C8E21245E}" name="Lote" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{683E82B8-B50D-4767-AA2F-7327EC16B03C}" name="Unidades" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{103F51FD-4980-4385-8737-6C121234FAAE}" name="Kg Bruto" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{1D36A2BF-02B3-4785-8579-39342D79E068}" name="Tara" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{90ECC13E-B58B-4180-8A1A-8808CCF6A5BD}" name="Kg Neto" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{64D76550-4432-4FE0-BDF8-015B9BCBB585}" name="Envasado" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F7EAB209-88B5-4D78-A4B2-A60F22AA2BF0}" name="Tabla3" displayName="Tabla3" ref="A28:H88" totalsRowShown="0" headerRowDxfId="72" headerRowBorderDxfId="71" tableBorderDxfId="70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F7EAB209-88B5-4D78-A4B2-A60F22AA2BF0}" name="Tabla3" displayName="Tabla3" ref="A28:H88" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A28:H88" xr:uid="{F7EAB209-88B5-4D78-A4B2-A60F22AA2BF0}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{528263D6-B342-4C1E-9AAD-290C4FCC42AE}" name="Descripcion"/>
@@ -4650,13 +4650,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>399</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:7" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="35"/>
@@ -4675,11 +4675,11 @@
     </row>
     <row r="3" spans="1:7" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A3" s="35"/>
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
       <c r="E3" s="36">
         <v>365</v>
       </c>
@@ -4846,7 +4846,7 @@
         <v>88</v>
       </c>
       <c r="B1" s="2">
-        <v>46142</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -6763,25 +6763,25 @@
         <v>88</v>
       </c>
       <c r="B1" s="2">
-        <v>46150</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="72" t="s">
         <v>234</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="74" t="s">
+      <c r="C3" s="73"/>
+      <c r="D3" s="72" t="s">
         <v>235</v>
       </c>
-      <c r="E3" s="75"/>
-      <c r="F3" s="74" t="s">
+      <c r="E3" s="73"/>
+      <c r="F3" s="72" t="s">
         <v>236</v>
       </c>
-      <c r="G3" s="75"/>
+      <c r="G3" s="73"/>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="19" t="s">
@@ -7435,13 +7435,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:7" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="35"/>
@@ -7460,11 +7460,11 @@
     </row>
     <row r="3" spans="1:7" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A3" s="35"/>
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
       <c r="E3" s="36">
         <v>365</v>
       </c>
@@ -9663,21 +9663,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>287</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:5" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A2" s="35"/>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="36">
         <v>21</v>
       </c>
@@ -9831,21 +9831,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>286</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:5" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A2" s="35"/>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="36">
         <v>5</v>
       </c>
@@ -9909,21 +9909,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>283</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:5" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A2" s="35"/>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="36">
         <v>65</v>
       </c>
@@ -10042,21 +10042,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:5" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A2" s="35"/>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="36">
         <f>10+35</f>
         <v>45</v>
@@ -10140,21 +10140,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="74" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="2" spans="1:5" ht="31.8" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A2" s="35"/>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="36">
         <v>150</v>
       </c>
@@ -10633,17 +10633,17 @@
         <v>88</v>
       </c>
       <c r="B1" s="2">
-        <v>46150</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="72" t="s">
         <v>258</v>
       </c>
-      <c r="C3" s="75"/>
+      <c r="C3" s="73"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="19" t="s">
@@ -10886,7 +10886,7 @@
         <v>88</v>
       </c>
       <c r="B1" s="2">
-        <v>46142</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>